<commit_message>
scenarios 5 and 6 are done
</commit_message>
<xml_diff>
--- a/test/test-cases/TestCases.xlsx
+++ b/test/test-cases/TestCases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORK\LEARNING\QA Engineer\Webdriver\e-commerce\test\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1FAA69C-4C07-401F-A0B0-4189C6387579}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{546CE75D-BBE4-464C-A74B-58F70CCB1CC2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -118,29 +118,6 @@
   </si>
   <si>
     <t>User is not registered</t>
-  </si>
-  <si>
-    <t>1. Go to https://automationexercise.com/
-2. Click on "Signup / login" link
-3. Go to "New User Signup!" form
-4. Input "uniquename" into name text input
-5. input email from test data into email text input
-6. Click on "Sign up" button
-7. Set "Mr." on radiobutton
-8. Input password from test data into password text input
-9. Set 01/01/2000 on date of birth
-10. Click on "Sign up for our newsletter!" select element
-11. Click on "Receive special offers from our partners!" select element
-12. Input "John" into First name text input
-13. Input "Doe" into Last name text input
-14. Input "123 Main St" into Adress text input
-15. Choose "United States" in Country list
-16. Input "NY" into State text input
-17. Input "Kingston" into City text input
-18. Input "12401" into Zipcode text input
-19. Input "0111111100" into Mobile Number text input
-20. Click on "Create Account" button
-21. Click on "Continue" button</t>
   </si>
   <si>
     <t>User is registered
@@ -341,6 +318,29 @@
 5. The payment page was opened
 6. The name was displayed without error message
 7. The error popup message was shown</t>
+  </si>
+  <si>
+    <t>1. Go to https://automationexercise.com/
+2. Click on "Signup / login" link
+3. Go to "New User Signup!" form
+4. Input "uniquename" into name text input
+5. input email from test data into email text input
+6. Click on "Sign up" button
+7. Set "Mr." on radiobutton
+8. Input password from test data into password text input
+9. Set 01/01/2000 on date of birth
+10. Click on "Sign up for our newsletter!" select element
+11. Click on "Receive special offers from our partners!" select element
+12. Input "John" into First name text input
+13. Input "Doe" into Last name text input
+14. Input "123 Main St" into Address text input
+15. Choose "United States" in Country list
+16. Input "NY" into State text input
+17. Input "Kingston" into City text input
+18. Input "12401" into Zipcode text input
+19. Input "0111111100" into Mobile Number text input
+20. Click on "Create Account" button
+21. Click on "Continue" button</t>
   </si>
 </sst>
 </file>
@@ -742,10 +742,10 @@
         <v>7</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>8</v>
@@ -760,7 +760,7 @@
         <v>13</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>9</v>
@@ -769,7 +769,7 @@
         <v>10</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>8</v>
@@ -784,16 +784,16 @@
         <v>14</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>30</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>11</v>
@@ -809,14 +809,14 @@
         <v>22</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>48</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>49</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>11</v>
@@ -831,14 +831,14 @@
         <v>21</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="4" t="s">
         <v>16</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>15</v>
@@ -853,16 +853,16 @@
         <v>17</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>33</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>34</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>11</v>
@@ -877,16 +877,16 @@
         <v>18</v>
       </c>
       <c r="C8" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>38</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>11</v>
@@ -901,14 +901,14 @@
         <v>19</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="4" t="s">
         <v>24</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>11</v>
@@ -923,16 +923,16 @@
         <v>20</v>
       </c>
       <c r="C10" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="E10" s="4" t="s">
+      <c r="F10" s="4" t="s">
         <v>46</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>47</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>8</v>
@@ -947,16 +947,16 @@
         <v>23</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E11" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>50</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>51</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>8</v>

</xml_diff>